<commit_message>
final production ready commit
</commit_message>
<xml_diff>
--- a/July_CEDH_Event/13th July CEDH Participant List.xlsx
+++ b/July_CEDH_Event/13th July CEDH Participant List.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cheah\Desktop\MTG-Tournament-Dashboard\July_CEDH_Event\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cheah\Documents\MTG-Dashboard\MTG-Tournament-Dashboard-AugmentCode\July_CEDH_Event\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBC6C98-2527-4F41-8A87-F54DE7F68395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C333EF98-2C13-4143-AD25-93A601C45E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t>Team Last Chance (TLC)</t>
   </si>
@@ -151,88 +151,124 @@
     <t>HandsomeMAN</t>
   </si>
   <si>
-    <t>e21e1</t>
-  </si>
-  <si>
-    <t>e21f2</t>
-  </si>
-  <si>
-    <t>32rr</t>
-  </si>
-  <si>
-    <t>r3</t>
-  </si>
-  <si>
-    <t>r3a</t>
-  </si>
-  <si>
-    <t>aa</t>
-  </si>
-  <si>
-    <t>qw</t>
-  </si>
-  <si>
-    <t>q3rq</t>
-  </si>
-  <si>
-    <t>qr3</t>
-  </si>
-  <si>
-    <t>ersgha</t>
-  </si>
-  <si>
-    <t>aw4a</t>
-  </si>
-  <si>
-    <t>4wt</t>
-  </si>
-  <si>
-    <t>yae</t>
-  </si>
-  <si>
-    <t>hdt</t>
-  </si>
-  <si>
-    <t>cxb</t>
-  </si>
-  <si>
-    <t>zf</t>
-  </si>
-  <si>
-    <t>sEg</t>
-  </si>
-  <si>
-    <t>sEGg</t>
-  </si>
-  <si>
-    <t>hea</t>
-  </si>
-  <si>
-    <t>hsr</t>
-  </si>
-  <si>
-    <t>cuk</t>
-  </si>
-  <si>
-    <t>kccm</t>
-  </si>
-  <si>
-    <t>fchm</t>
-  </si>
-  <si>
-    <t>fcft</t>
-  </si>
-  <si>
-    <t>hxtfht</t>
-  </si>
-  <si>
-    <t>txh</t>
-  </si>
-  <si>
-    <t>xth</t>
-  </si>
-  <si>
-    <t>hrtx</t>
+    <t>Laksa &amp; Logic</t>
+  </si>
+  <si>
+    <t>Wei Ming</t>
+  </si>
+  <si>
+    <t>Jonathan</t>
+  </si>
+  <si>
+    <t>Samuel</t>
+  </si>
+  <si>
+    <t>Yi Xuan</t>
+  </si>
+  <si>
+    <t>Kopi C Kosong</t>
+  </si>
+  <si>
+    <t>Jun Hao</t>
+  </si>
+  <si>
+    <t>Kelvin</t>
+  </si>
+  <si>
+    <t>Wei Jie</t>
+  </si>
+  <si>
+    <t>Amanda</t>
+  </si>
+  <si>
+    <t>System Override</t>
+  </si>
+  <si>
+    <t>Ming Han</t>
+  </si>
+  <si>
+    <t>Shaun</t>
+  </si>
+  <si>
+    <t>Tiffany</t>
+  </si>
+  <si>
+    <t>Aloysius</t>
+  </si>
+  <si>
+    <t>West Mall Warriors</t>
+  </si>
+  <si>
+    <t>Zhi Cong</t>
+  </si>
+  <si>
+    <t>Darren</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Benjamin</t>
+  </si>
+  <si>
+    <t>Infinite Loop</t>
+  </si>
+  <si>
+    <t>Wen Long</t>
+  </si>
+  <si>
+    <t>Isaac</t>
+  </si>
+  <si>
+    <t>Rachel</t>
+  </si>
+  <si>
+    <t>Khairul</t>
+  </si>
+  <si>
+    <t>Chicken Rice lobang</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Nicholas</t>
+  </si>
+  <si>
+    <t>Zi Wei</t>
+  </si>
+  <si>
+    <t>Hafiz</t>
+  </si>
+  <si>
+    <t>Error 404 Found</t>
+  </si>
+  <si>
+    <t>Jian Hong</t>
+  </si>
+  <si>
+    <t>Lewis</t>
+  </si>
+  <si>
+    <t>Stanley</t>
+  </si>
+  <si>
+    <t>Wei Ting</t>
+  </si>
+  <si>
+    <t>The Git Committers</t>
+  </si>
+  <si>
+    <t>Leon</t>
+  </si>
+  <si>
+    <t>Marcus</t>
+  </si>
+  <si>
+    <t>Sheng</t>
+  </si>
+  <si>
+    <t>Bala</t>
   </si>
 </sst>
 </file>
@@ -559,29 +595,29 @@
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="1">
-        <v>1111</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2222</v>
-      </c>
-      <c r="K1" s="1">
-        <v>3333</v>
-      </c>
-      <c r="L1" s="1">
-        <v>4444</v>
-      </c>
-      <c r="M1" s="1">
-        <v>5555</v>
-      </c>
-      <c r="N1" s="1">
-        <v>6666</v>
-      </c>
-      <c r="O1" s="1">
-        <v>7777</v>
-      </c>
-      <c r="P1" s="1">
-        <v>8888</v>
+      <c r="I1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -609,29 +645,29 @@
       <c r="H2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="2">
-        <v>123123</v>
+      <c r="I2" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="L2" s="2">
-        <v>4</v>
+        <v>54</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -659,29 +695,29 @@
       <c r="H3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="2">
-        <v>2312</v>
+      <c r="I3" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -709,29 +745,29 @@
       <c r="H4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="2">
-        <v>12312313</v>
+      <c r="I4" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -760,28 +796,28 @@
         <v>33</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>